<commit_message>
fix(finance): make forecast horizon truthful
</commit_message>
<xml_diff>
--- a/product_release/work_items/financial-analysis/SpeakSharp_Updated_Financial_Model_2026-09-05.xlsx
+++ b/product_release/work_items/financial-analysis/SpeakSharp_Updated_Financial_Model_2026-09-05.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re62df55e24c64533"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rac304b7c2b3f4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Comparison" sheetId="3" r:id="R090b754b61514659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini Options" sheetId="4" r:id="R8395bc34b0584987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior Models" sheetId="5" r:id="Rbd22be7ec68e4361"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast 12M" sheetId="6" r:id="R7f3e5b6f689647da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" r:id="R87c2de35bfa74f2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Re68ec17416d84ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R66c9e98c8fdd4994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4f3f69d6fdad4600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R14029db5ee3a45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Comparison" sheetId="3" r:id="R41a3ac2b2d084154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini Options" sheetId="4" r:id="R454a39665b8b49ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior Models" sheetId="5" r:id="R8f2efaa60cb941c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast 12M" sheetId="6" r:id="Rb948f799c6f74f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" r:id="R768e7cafd7984b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R76d4dec6f0fb4e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R7f4c556edf2e4216"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1444,7 +1444,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0068453e2e2548d1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcfe53f46d58b45f2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1479,7 +1479,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf91b44f22d1347bf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re3732fed6ef94946"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1514,7 +1514,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb61df472bb994851"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfcb461268c614c1b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2904,7 +2904,7 @@
     <x:mergeCell ref="A32:H34"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2faf91e73e5c497b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bdac0146f4a4bb6"/>
 </x:worksheet>
 </file>
 
@@ -3042,22 +3042,23 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="149" t="str">
-        <x:v>Forecast months</x:v>
+        <x:v>Forecast horizon</x:v>
       </x:c>
       <x:c r="B7" s="156" t="n">
+        <x:f>COLUMNS('Forecast 12M'!B3:M3)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C7" s="149" t="str">
         <x:v>months</x:v>
       </x:c>
       <x:c r="D7" s="149" t="str">
-        <x:v>Input</x:v>
+        <x:v>Formula</x:v>
       </x:c>
       <x:c r="E7" s="149" t="str">
-        <x:v>Management horizon</x:v>
+        <x:v>Count of forecast month columns</x:v>
       </x:c>
       <x:c r="F7" s="149" t="str">
-        <x:v>12-month base model</x:v>
+        <x:v>Fixed layout; extend Forecast 12M and this formula together</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3728,7 +3729,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb34fdf70489d4172"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9203f3590f4472"/>
 </x:worksheet>
 </file>
 
@@ -4501,7 +4502,7 @@
     <x:mergeCell ref="A21:G21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7acc7fd343e4298"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R479ec53ecb9146d0"/>
 </x:worksheet>
 </file>
 
@@ -8129,7 +8130,7 @@
     <x:mergeCell ref="A32:M32"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5eb82187a3af41bf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7af21e534014968"/>
 </x:worksheet>
 </file>
 
@@ -9102,13 +9103,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="204" t="str">
-        <x:f>IF(COUNTIF(F5:F15,"FAIL")+COUNTIF(F20:F22,"FAIL")=0,"MODEL STATUS: PASS","MODEL STATUS: FAIL")</x:f>
+        <x:f>IF(COUNTIF(F5:F15,"FAIL")+COUNTIF(F20:F23,"FAIL")=0,"MODEL STATUS: PASS","MODEL STATUS: FAIL")</x:f>
         <x:v>MODEL STATUS: PASS</x:v>
       </x:c>
       <x:c r="B18" s="204"/>
       <x:c r="C18" s="124"/>
       <x:c r="D18" s="205" t="str">
-        <x:v>Financial audit completed: historical claims reconciled; trial and paid coaching usage included; Gemini's 2027 price step included; fixed and variable costs separated; paid CAC shown separately. PASS confirms formula consistency, not commercial validation.</x:v>
+        <x:v>Financial audit completed: historical claims reconciled; trial and paid coaching usage included; Gemini's 2027 price step included; fixed and variable costs separated; paid CAC shown separately; forecast horizon tied to the fixed 12-month layout. PASS confirms formula consistency, not commercial validation.</x:v>
       </x:c>
       <x:c r="E18" s="205" t="str">
         <x:v>Financial audit completed: historical claims reconciled, 30-day trial timing separated from the old immediate-paid ramp, Gemini's 2027 price step included, fixed and variable costs separated, and paid CAC shown as a separate scenario rather than hidden from profit.</x:v>
@@ -9216,6 +9217,33 @@
       </x:c>
       <x:c r="G22" t="str">
         <x:v>Forecast 12M B21 / 500 active trials</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Forecast horizon matches forecast columns</x:v>
+      </x:c>
+      <x:c r="B23" t="n">
+        <x:f>'Assumptions'!B7</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:f>COLUMNS('Forecast 12M'!B3:M3)</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D23" t="n">
+        <x:f>B23-C23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:f>IF(ABS(D23)&lt;=E23,"OK","FAIL")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Assumptions B7 / Forecast 12M B:M</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix(finance): mark fixed horizon as formula
</commit_message>
<xml_diff>
--- a/product_release/work_items/financial-analysis/SpeakSharp_Updated_Financial_Model_2026-09-05.xlsx
+++ b/product_release/work_items/financial-analysis/SpeakSharp_Updated_Financial_Model_2026-09-05.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4f3f69d6fdad4600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R14029db5ee3a45b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Comparison" sheetId="3" r:id="R41a3ac2b2d084154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini Options" sheetId="4" r:id="R454a39665b8b49ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior Models" sheetId="5" r:id="R8f2efaa60cb941c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast 12M" sheetId="6" r:id="Rb948f799c6f74f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" r:id="R768e7cafd7984b5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R76d4dec6f0fb4e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R7f4c556edf2e4216"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1ef1ece6c71f4653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R3da7e09046e54d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Comparison" sheetId="3" r:id="Rb358a995d40540aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini Options" sheetId="4" r:id="Rd6a409a3af034156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prior Models" sheetId="5" r:id="R41e2daf4fa7840f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast 12M" sheetId="6" r:id="R6f6048665ee14bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="7" r:id="R607fda8ac3ea4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="Rc18e75ac24534203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R3da6e1052967472b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -276,6 +276,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE8F5EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2FF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -352,7 +357,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="206">
+  <x:cellXfs count="207">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -898,6 +903,9 @@
     <x:xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="25" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1444,7 +1452,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcfe53f46d58b45f2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdaf6d83bde564f51"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1479,7 +1487,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re3732fed6ef94946"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R947fd4d34adb46c3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1514,7 +1522,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfcb461268c614c1b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a1fc6054bdc4e5b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2904,7 +2912,7 @@
     <x:mergeCell ref="A32:H34"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bdac0146f4a4bb6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a275f92841b4371"/>
 </x:worksheet>
 </file>
 
@@ -3044,7 +3052,7 @@
       <x:c r="A7" s="149" t="str">
         <x:v>Forecast horizon</x:v>
       </x:c>
-      <x:c r="B7" s="156" t="n">
+      <x:c r="B7" s="206" t="n">
         <x:f>COLUMNS('Forecast 12M'!B3:M3)</x:f>
         <x:v>12</x:v>
       </x:c>
@@ -3729,7 +3737,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9203f3590f4472"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a2f28c579f14ac4"/>
 </x:worksheet>
 </file>
 
@@ -4502,7 +4510,7 @@
     <x:mergeCell ref="A21:G21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R479ec53ecb9146d0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd4c0c9e06d94b00"/>
 </x:worksheet>
 </file>
 
@@ -8130,7 +8138,7 @@
     <x:mergeCell ref="A32:M32"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7af21e534014968"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recf8fe525c2c4c4b"/>
 </x:worksheet>
 </file>
 

</xml_diff>